<commit_message>
feat: update books from Excel — 556 books (+12 new)
</commit_message>
<xml_diff>
--- a/Книги.xlsx
+++ b/Книги.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dmitrypotekhin/Downloads/dmpotekhin.github.io/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF84D64C-7B01-C04F-AD4D-2F1AA0AFCADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EEE91FA-6457-4248-847C-702C9EF37F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="16000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1628" uniqueCount="892">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1667" uniqueCount="914">
   <si>
     <t>Борис Акунин</t>
   </si>
@@ -2700,6 +2700,72 @@
   </si>
   <si>
     <t>Elisabeth Hendrickson</t>
+  </si>
+  <si>
+    <t>Как работает музыка</t>
+  </si>
+  <si>
+    <t>Дэвид Бирн</t>
+  </si>
+  <si>
+    <t>Роджер Кроули</t>
+  </si>
+  <si>
+    <t>Завоеватели Как Португальцы первую мировую империю</t>
+  </si>
+  <si>
+    <t>Феникс  Роман о том, как Devops  меняет бизнес к лучшему</t>
+  </si>
+  <si>
+    <t>Ким Джин</t>
+  </si>
+  <si>
+    <t>Coca-Cola История великого напитка</t>
+  </si>
+  <si>
+    <t>Марк Пендерграст</t>
+  </si>
+  <si>
+    <t>Законы человеческой природы</t>
+  </si>
+  <si>
+    <t>Джесси Инчаспе</t>
+  </si>
+  <si>
+    <t>Богиня Глкозы</t>
+  </si>
+  <si>
+    <t>Кэрол Дуэк</t>
+  </si>
+  <si>
+    <t>Гибкое сознание</t>
+  </si>
+  <si>
+    <t>Виктор Гюго</t>
+  </si>
+  <si>
+    <t>Человек, который смеется</t>
+  </si>
+  <si>
+    <t>Собор парижской Богоматери</t>
+  </si>
+  <si>
+    <t>Отверженные</t>
+  </si>
+  <si>
+    <t>Человек в поисках смысла</t>
+  </si>
+  <si>
+    <t>Ускоряйся Наука Devops</t>
+  </si>
+  <si>
+    <t>Николь Форсгрен</t>
+  </si>
+  <si>
+    <t>Непрерывный рефакторинг</t>
+  </si>
+  <si>
+    <t>Дмитрий Голицын</t>
   </si>
 </sst>
 </file>
@@ -3001,7 +3067,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:U552"/>
+  <dimension ref="A1:U557"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -9796,8 +9862,148 @@
         <v>2</v>
       </c>
     </row>
-    <row r="552" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B552" s="5"/>
+    <row r="545" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A545" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="B545" s="4" t="s">
+        <v>892</v>
+      </c>
+      <c r="C545" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="546" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A546" s="4" t="s">
+        <v>894</v>
+      </c>
+      <c r="B546" s="4" t="s">
+        <v>895</v>
+      </c>
+      <c r="C546" s="5" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="547" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A547" s="4" t="s">
+        <v>897</v>
+      </c>
+      <c r="B547" s="4" t="s">
+        <v>896</v>
+      </c>
+      <c r="C547" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="548" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A548" s="4" t="s">
+        <v>899</v>
+      </c>
+      <c r="B548" s="4" t="s">
+        <v>898</v>
+      </c>
+      <c r="C548" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="549" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A549" s="4" t="s">
+        <v>554</v>
+      </c>
+      <c r="B549" s="4" t="s">
+        <v>900</v>
+      </c>
+      <c r="C549" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="550" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A550" s="4" t="s">
+        <v>901</v>
+      </c>
+      <c r="B550" s="4" t="s">
+        <v>902</v>
+      </c>
+      <c r="C550" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="551" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A551" s="4" t="s">
+        <v>903</v>
+      </c>
+      <c r="B551" s="4" t="s">
+        <v>904</v>
+      </c>
+      <c r="C551" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="552" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A552" s="4" t="s">
+        <v>905</v>
+      </c>
+      <c r="B552" s="4" t="s">
+        <v>906</v>
+      </c>
+      <c r="C552" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="553" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A553" s="4" t="s">
+        <v>905</v>
+      </c>
+      <c r="B553" s="4" t="s">
+        <v>907</v>
+      </c>
+      <c r="C553" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="554" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A554" s="4" t="s">
+        <v>905</v>
+      </c>
+      <c r="B554" s="4" t="s">
+        <v>908</v>
+      </c>
+      <c r="C554" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="555" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A555" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="B555" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="C555" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="556" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A556" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="B556" s="4" t="s">
+        <v>910</v>
+      </c>
+      <c r="C556" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="557" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A557" s="4" t="s">
+        <v>913</v>
+      </c>
+      <c r="B557" s="4" t="s">
+        <v>912</v>
+      </c>
+      <c r="C557" s="1" t="s">
+        <v>107</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:C506" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
feat: update books from Excel — 562 books (+6 new)
New books with notes:
- На пенсию в 35 (Анар Бабаев)
- 7 сил Основы бизнес-стратеги (Гамильтон Хелмер)
- Никогда-нибудь (Елена Резанова)
- Автономное выживание (Игорь Молодан)
- Власть и прогресс (Дарон Аджемоглу)
- Немцы после войны (Николай Власов)
</commit_message>
<xml_diff>
--- a/Книги.xlsx
+++ b/Книги.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dmitrypotekhin/Downloads/dmpotekhin.github.io/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EEE91FA-6457-4248-847C-702C9EF37F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A41D25D4-2550-964F-904D-89AF4DC6095A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="16000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1667" uniqueCount="914">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1685" uniqueCount="926">
   <si>
     <t>Борис Акунин</t>
   </si>
@@ -2766,6 +2766,42 @@
   </si>
   <si>
     <t>Дмитрий Голицын</t>
+  </si>
+  <si>
+    <t>На пенсию в 35</t>
+  </si>
+  <si>
+    <t>Анар Бабаев</t>
+  </si>
+  <si>
+    <t>Гамильтон Хелмер</t>
+  </si>
+  <si>
+    <t>7 сил Основы бизнес-стратеги</t>
+  </si>
+  <si>
+    <t>Елена Резанова</t>
+  </si>
+  <si>
+    <t>Никогда-нибудь. Как выйти из тупика и найти себя</t>
+  </si>
+  <si>
+    <t>Автономное выживание</t>
+  </si>
+  <si>
+    <t>Игорь Молодан</t>
+  </si>
+  <si>
+    <t>Власть и прогресс</t>
+  </si>
+  <si>
+    <t>Дарон Аджемоглу</t>
+  </si>
+  <si>
+    <t>Немцы после войны: Как Западной Германии удалось преодолеть нацизм</t>
+  </si>
+  <si>
+    <t>Николай Власов</t>
   </si>
 </sst>
 </file>
@@ -3067,7 +3103,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:U557"/>
+  <dimension ref="A1:U563"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -10005,6 +10041,72 @@
         <v>107</v>
       </c>
     </row>
+    <row r="558" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A558" s="4" t="s">
+        <v>915</v>
+      </c>
+      <c r="B558" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="C558" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="559" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A559" s="4" t="s">
+        <v>916</v>
+      </c>
+      <c r="B559" s="4" t="s">
+        <v>917</v>
+      </c>
+      <c r="C559" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="560" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A560" s="4" t="s">
+        <v>918</v>
+      </c>
+      <c r="B560" s="4" t="s">
+        <v>919</v>
+      </c>
+      <c r="C560" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="561" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A561" s="4" t="s">
+        <v>921</v>
+      </c>
+      <c r="B561" s="4" t="s">
+        <v>920</v>
+      </c>
+      <c r="C561" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="562" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A562" s="4" t="s">
+        <v>923</v>
+      </c>
+      <c r="B562" s="4" t="s">
+        <v>922</v>
+      </c>
+      <c r="C562" s="5" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="563" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A563" s="4" t="s">
+        <v>925</v>
+      </c>
+      <c r="B563" s="4" t="s">
+        <v>924</v>
+      </c>
+      <c r="C563" s="5" t="s">
+        <v>168</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C506" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>